<commit_message>
Add evidence references to all attribute columns B–O
Each application sample on the Application + Attribute Testing tab now
lists its supporting BSI.IT.6.C7.3 evidence files under every column from
IT DR exercise name through Results Documented in BCMS, sourced from the
Evidence Map tab. Column F widened and row heights adjusted to fit.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017gG3mo6UXrWCJH3UHBXjTp
</commit_message>
<xml_diff>
--- a/BSI.IT.6.C7.3_E00_Workpaper_DR_DIV_INTEGRATED_APPLICATION_Evidence_Mapped.xlsx
+++ b/BSI.IT.6.C7.3_E00_Workpaper_DR_DIV_INTEGRATED_APPLICATION_Evidence_Mapped.xlsx
@@ -439,7 +439,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -648,6 +648,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -2121,7 +2124,7 @@
     <col width="38" customWidth="1" style="70" min="3" max="3"/>
     <col width="34" customWidth="1" style="70" min="4" max="4"/>
     <col width="48" customWidth="1" style="70" min="5" max="5"/>
-    <col width="12" customWidth="1" style="70" min="6" max="6"/>
+    <col width="34" customWidth="1" style="70" min="6" max="6"/>
     <col width="34" customWidth="1" style="70" min="7" max="7"/>
     <col width="38" customWidth="1" style="70" min="8" max="8"/>
     <col width="46" customWidth="1" style="70" min="9" max="9"/>
@@ -2310,62 +2313,105 @@
       </c>
       <c r="C5" s="45" t="inlineStr">
         <is>
-          <t>ACH Express</t>
+          <t>ACH Express
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 3)
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E03 – All Data Integrity Validation Testing FV (row 47)
+• E04 – BCiC Screenshot for Data Integrity Validation report (screen of the report; record on later page)</t>
         </is>
       </c>
       <c r="D5" s="45" t="inlineStr">
         <is>
-          <t>Andreina De Stefano</t>
+          <t>Andreina De Stefano
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 47)
+• E04 – BCiC Screenshot for Data Integrity Validation report (screen of the report; record on later page)</t>
         </is>
       </c>
       <c r="E5" s="45" t="inlineStr">
         <is>
-          <t>11/15/2025</t>
+          <t>11/15/2025
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 47)
+• E04 – BCiC Screenshot for Data Integrity Validation report (screen of the report; record on later page)
+• E09 – RE: Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi</t>
         </is>
       </c>
       <c r="F5" s="45" t="inlineStr">
         <is>
-          <t>Claudia Romero</t>
+          <t>Claudia Romero
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 47)
+• E04 – BCiC Screenshot for Data Integrity Validation report (screen of the report; record on later page)</t>
         </is>
       </c>
       <c r="G5" s="45" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>05/05/2026
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 47)
+• E04 – BCiC Screenshot for Data Integrity Validation report (screen of the report; record on later page)</t>
         </is>
       </c>
       <c r="H5" s="45" t="inlineStr">
         <is>
-          <t>FED Inclearing (ACH &amp; Cash Letters) ACH Express Data Integrity Validation (DIV) Procedure</t>
+          <t>FED Inclearing (ACH &amp; Cash Letters) ACH Express Data Integrity Validation (DIV) Procedure
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 47) – 'Data Integrity Validation Procedures' column
+• E04 – BCiC Screenshot for Data Integrity Validation report (screen of the report; record on later page)</t>
         </is>
       </c>
       <c r="I5" s="45" t="inlineStr">
         <is>
-          <t>Yes – Client Back Office group-level approval is evidenced by Claudia Romero’s 05/05/2026 approval of the backup/restore test results. Scope mapping ties ACH Express to Client Back Office.</t>
+          <t>Yes – Client Back Office group-level approval is evidenced by Claudia Romero’s 05/05/2026 approval of the backup/restore test results. Scope mapping ties ACH Express to Client Back Office.
+See BSI.IT.6.C7.3 evidence folder:
+• E09 – RE: Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi
+→ Claudia Romero – "Approved" 05/05/2026 (Client Back Office backup/restore results incl. ACH Express)</t>
         </is>
       </c>
       <c r="J5" s="46" t="inlineStr">
         <is>
-          <t>VALID – BCIC evidence confirmed. The BC in the Cloud 'Applications In Scope for DR Test BSI' view directly displays this application as in scope, and the BCIC Data Integrity Validation Testing screen corroborates the source report used for the detailed DIV population. The detailed source export contains this application's DIV record and approval fields.</t>
+          <t>VALID – BCIC evidence confirmed. The BC in the Cloud 'Applications In Scope for DR Test BSI' view directly displays this application as in scope, and the BCIC Data Integrity Validation Testing screen corroborates the source report used for the detailed DIV population. The detailed source export contains this application's DIV record and approval fields.
+See BSI.IT.6.C7.3 evidence folder:
+• E04 – BCiC Screenshot for Data Integrity Validation report
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E03 – All Data Integrity Validation Testing FV
+• E01 – Applications In Scope for DR Test BSI (13)</t>
         </is>
       </c>
       <c r="K5" s="80" t="inlineStr">
         <is>
-          <t>PASS – The application is included in the annual DR/Data Integrity Validation testing population for the review period, supported by the documented 2025/2026 DR exercises and the BCiC testing records.</t>
+          <t>PASS – The application is included in the annual DR/Data Integrity Validation testing population for the review period, supported by the documented 2025/2026 DR exercises and the BCiC testing records.
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 3) – Exercise Date / 2025-2026 DR Test Scope
+• E03 – All Data Integrity Validation Testing FV (row 47) – Business Data Validation Date / Last App DR Test Date</t>
         </is>
       </c>
       <c r="L5" s="80" t="inlineStr">
         <is>
-          <t>PASS – IT DR facilitated the Data Integrity Validation process and the designated business-line tester performed the validation during the DR exercise. The application record contains the validation date/results.</t>
+          <t>PASS – IT DR facilitated the Data Integrity Validation process and the designated business-line tester performed the validation during the DR exercise. The application record contains the validation date/results.
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 47) – Y/N Format, Headers, Content = Y
+• E09 – RE: Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi</t>
         </is>
       </c>
       <c r="M5" s="80" t="inlineStr">
         <is>
-          <t>PASS – ACH Express is supported as in scope through the BCM/BIA process led by Elizabeth Noda and corroborated by the BCiC/workpaper scope population. A separate Michael Sacilotto approval list is not required for the evidenced process. See Management_Attestation folder</t>
+          <t>PASS – ACH Express is supported as in scope through the BCM/BIA process led by Elizabeth Noda and corroborated by the BCiC/workpaper scope population. A separate Michael Sacilotto approval list is not required for the evidenced process. See Management_Attestation folder
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 3)
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E05 – IT BIA Results Review and preparation for DR
+• E06 – IT BIA Results Review and preparation for DR 1 (1)</t>
         </is>
       </c>
       <c r="N5" s="80" t="inlineStr">
         <is>
-          <t>PASS – Business-line review/approval is supported by the BCiC manager approval fields for Claudia Romero dated 05/05/2026. Supplemental approval emails/attestations are used where available.</t>
+          <t>PASS – Business-line review/approval is supported by the BCiC manager approval fields for Claudia Romero dated 05/05/2026. Supplemental approval emails/attestations are used where available.
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 47) – Department Manager / Approval Date
+• E09 – RE: Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi</t>
         </is>
       </c>
       <c r="O5" s="80" t="inlineStr">
@@ -2447,7 +2493,7 @@
       <c r="BL5" s="61" t="n"/>
       <c r="BM5" s="61" t="n"/>
     </row>
-    <row r="6" ht="150" customFormat="1" customHeight="1" s="39">
+    <row r="6" ht="264" customFormat="1" customHeight="1" s="39">
       <c r="A6" s="45" t="n">
         <v>1867</v>
       </c>
@@ -2462,62 +2508,105 @@
       </c>
       <c r="C6" s="45" t="inlineStr">
         <is>
-          <t>FedExport - BSI</t>
+          <t>FedExport - BSI
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 19)
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E03 – All Data Integrity Validation Testing FV (row 9)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
         </is>
       </c>
       <c r="D6" s="45" t="inlineStr">
         <is>
-          <t>Andreina De Stefano</t>
+          <t>Andreina De Stefano
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 9)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
         </is>
       </c>
       <c r="E6" s="45" t="inlineStr">
         <is>
-          <t>11/15/2025</t>
+          <t>11/15/2025
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 9)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)
+• E09 – RE: Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi</t>
         </is>
       </c>
       <c r="F6" s="45" t="inlineStr">
         <is>
-          <t>Claudia Romero</t>
+          <t>Claudia Romero
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 9)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
         </is>
       </c>
       <c r="G6" s="45" t="inlineStr">
         <is>
-          <t>06/05/2026</t>
+          <t>06/05/2026
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 9)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
         </is>
       </c>
       <c r="H6" s="45" t="inlineStr">
         <is>
-          <t>FED Inclearing (ACH &amp; Cash Letters) FedExport - BSI Data Integrity Validation (DIV) Procedure</t>
+          <t>FED Inclearing (ACH &amp; Cash Letters) FedExport - BSI Data Integrity Validation (DIV) Procedure
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 9) – 'Data Integrity Validation Procedures' column
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
         </is>
       </c>
       <c r="I6" s="45" t="inlineStr">
         <is>
-          <t>Yes – Client Back Office group-level approval is evidenced by Claudia Romero’s 05/05/2026 approval of the backup/restore test results. Scope mapping ties FedExport - BSI to Client Back Office.</t>
+          <t>Yes – Client Back Office group-level approval is evidenced by Claudia Romero’s 05/05/2026 approval of the backup/restore test results. Scope mapping ties FedExport - BSI to Client Back Office.
+See BSI.IT.6.C7.3 evidence folder:
+• E09 – RE: Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi
+→ Claudia Romero – "Approved" 05/05/2026 (Client Back Office incl. FedExport)</t>
         </is>
       </c>
       <c r="J6" s="46" t="inlineStr">
         <is>
-          <t>VALID – BCIC evidence confirmed. The BC in the Cloud 'Data Integrity Validation Testing' screen directly displays this application and the control fields for Business Data Validation Date, Department Manager, Department Manager Approval Date, and Y/N Format, Headers, and Content. The detailed BCIC source export supports the full application record.</t>
+          <t>VALID – BCIC evidence confirmed. The BC in the Cloud 'Data Integrity Validation Testing' screen directly displays this application and the control fields for Business Data Validation Date, Department Manager, Department Manager Approval Date, and Y/N Format, Headers, and Content. The detailed BCIC source export supports the full application record.
+See BSI.IT.6.C7.3 evidence folder:
+• E04 – BCiC Screenshot for Data Integrity Validation report
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E03 – All Data Integrity Validation Testing FV
+• E01 – Applications In Scope for DR Test BSI (13)</t>
         </is>
       </c>
       <c r="K6" s="80" t="inlineStr">
         <is>
-          <t>PASS – The application is included in the annual DR/Data Integrity Validation testing population for the review period, supported by the documented 2025/2026 DR exercises and the BCiC testing records.</t>
+          <t>PASS – The application is included in the annual DR/Data Integrity Validation testing population for the review period, supported by the documented 2025/2026 DR exercises and the BCiC testing records.
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 19) – Exercise Date / 2025-2026 DR Test Scope
+• E03 – All Data Integrity Validation Testing FV (row 9) – Business Data Validation Date / Last App DR Test Date</t>
         </is>
       </c>
       <c r="L6" s="80" t="inlineStr">
         <is>
-          <t>PASS – IT DR facilitated the Data Integrity Validation process and the designated business-line tester performed the validation during the DR exercise. The application record contains the validation date/results.</t>
+          <t>PASS – IT DR facilitated the Data Integrity Validation process and the designated business-line tester performed the validation during the DR exercise. The application record contains the validation date/results.
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 9) – Y/N Format, Headers, Content = Y
+• E09 – RE: Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi</t>
         </is>
       </c>
       <c r="M6" s="80" t="inlineStr">
         <is>
-          <t>PASS – FedExport - BSI is supported as in scope through the BCM/BIA process led by Elizabeth Noda and corroborated by the BCiC/workpaper scope population. A separate Michael Sacilotto approval list is not required for the evidenced process. See Management_Attestation folder</t>
+          <t>PASS – FedExport - BSI is supported as in scope through the BCM/BIA process led by Elizabeth Noda and corroborated by the BCiC/workpaper scope population. A separate Michael Sacilotto approval list is not required for the evidenced process. See Management_Attestation folder
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 19)
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E05 – IT BIA Results Review and preparation for DR
+• E06 – IT BIA Results Review and preparation for DR 1 (1)</t>
         </is>
       </c>
       <c r="N6" s="80" t="inlineStr">
         <is>
-          <t>PASS – Business-line review/approval is supported by the BCiC manager approval fields for Claudia Romero dated 06/05/2026. Supplemental approval emails/attestations are used where available.</t>
+          <t>PASS – Business-line review/approval is supported by the BCiC manager approval fields for Claudia Romero dated 06/05/2026. Supplemental approval emails/attestations are used where available.
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 9) – Department Manager / Approval Date
+• E09 – RE: Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi</t>
         </is>
       </c>
       <c r="O6" s="80" t="inlineStr">
@@ -2599,7 +2688,7 @@
       <c r="BL6" s="61" t="n"/>
       <c r="BM6" s="61" t="n"/>
     </row>
-    <row r="7" ht="150" customFormat="1" customHeight="1" s="39">
+    <row r="7" ht="264" customFormat="1" customHeight="1" s="39">
       <c r="A7" s="45" t="n">
         <v>1868</v>
       </c>
@@ -2614,62 +2703,105 @@
       </c>
       <c r="C7" s="45" t="inlineStr">
         <is>
-          <t>FedImport - BSI</t>
+          <t>FedImport - BSI
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 20)
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E03 – All Data Integrity Validation Testing FV (row 10)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
         </is>
       </c>
       <c r="D7" s="45" t="inlineStr">
         <is>
-          <t>Andreina De Stefano</t>
+          <t>Andreina De Stefano
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 10)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
         </is>
       </c>
       <c r="E7" s="45" t="inlineStr">
         <is>
-          <t>11/15/2025</t>
+          <t>11/15/2025
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 10)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)
+• E09 – RE: Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi</t>
         </is>
       </c>
       <c r="F7" s="45" t="inlineStr">
         <is>
-          <t>Claudia Romero</t>
+          <t>Claudia Romero
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 10)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
         </is>
       </c>
       <c r="G7" s="45" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>05/05/2026
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 10)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
         </is>
       </c>
       <c r="H7" s="45" t="inlineStr">
         <is>
-          <t>FED Inclearing (ACH &amp; Cash Letters) FedImport - BSI Data Integrity Validation (DIV) Procedure</t>
+          <t>FED Inclearing (ACH &amp; Cash Letters) FedImport - BSI Data Integrity Validation (DIV) Procedure
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 10) – 'Data Integrity Validation Procedures' column
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
         </is>
       </c>
       <c r="I7" s="45" t="inlineStr">
         <is>
-          <t>Yes – Client Back Office group-level approval is evidenced by Claudia Romero’s 05/05/2026 approval of the backup/restore test results. Scope mapping ties FedImport - BSI to Client Back Office.</t>
+          <t>Yes – Client Back Office group-level approval is evidenced by Claudia Romero’s 05/05/2026 approval of the backup/restore test results. Scope mapping ties FedImport - BSI to Client Back Office.
+See BSI.IT.6.C7.3 evidence folder:
+• E09 – RE: Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi
+→ Claudia Romero – "Approved" 05/05/2026 (Client Back Office incl. FedImport)</t>
         </is>
       </c>
       <c r="J7" s="46" t="inlineStr">
         <is>
-          <t>VALID – BCIC evidence confirmed. The BC in the Cloud 'Data Integrity Validation Testing' screen directly displays this application and the control fields for Business Data Validation Date, Department Manager, Department Manager Approval Date, and Y/N Format, Headers, and Content. The detailed BCIC source export supports the full application record.</t>
+          <t>VALID – BCIC evidence confirmed. The BC in the Cloud 'Data Integrity Validation Testing' screen directly displays this application and the control fields for Business Data Validation Date, Department Manager, Department Manager Approval Date, and Y/N Format, Headers, and Content. The detailed BCIC source export supports the full application record.
+See BSI.IT.6.C7.3 evidence folder:
+• E04 – BCiC Screenshot for Data Integrity Validation report
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E03 – All Data Integrity Validation Testing FV
+• E01 – Applications In Scope for DR Test BSI (13)</t>
         </is>
       </c>
       <c r="K7" s="80" t="inlineStr">
         <is>
-          <t>PASS – The application is included in the annual DR/Data Integrity Validation testing population for the review period, supported by the documented 2025/2026 DR exercises and the BCiC testing records.</t>
+          <t>PASS – The application is included in the annual DR/Data Integrity Validation testing population for the review period, supported by the documented 2025/2026 DR exercises and the BCiC testing records.
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 20) – Exercise Date / 2025-2026 DR Test Scope
+• E03 – All Data Integrity Validation Testing FV (row 10) – Business Data Validation Date / Last App DR Test Date</t>
         </is>
       </c>
       <c r="L7" s="80" t="inlineStr">
         <is>
-          <t>PASS – IT DR facilitated the Data Integrity Validation process and the designated business-line tester performed the validation during the DR exercise. The application record contains the validation date/results.</t>
+          <t>PASS – IT DR facilitated the Data Integrity Validation process and the designated business-line tester performed the validation during the DR exercise. The application record contains the validation date/results.
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 10) – Y/N Format, Headers, Content = Y
+• E09 – RE: Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi</t>
         </is>
       </c>
       <c r="M7" s="80" t="inlineStr">
         <is>
-          <t>PASS – FedImport - BSI is supported as in scope through the BCM/BIA process led by Elizabeth Noda and corroborated by the BCiC/workpaper scope population. A separate Michael Sacilotto approval list is not required for the evidenced process. See Management_Attestation folder</t>
+          <t>PASS – FedImport - BSI is supported as in scope through the BCM/BIA process led by Elizabeth Noda and corroborated by the BCiC/workpaper scope population. A separate Michael Sacilotto approval list is not required for the evidenced process. See Management_Attestation folder
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 20)
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E05 – IT BIA Results Review and preparation for DR
+• E06 – IT BIA Results Review and preparation for DR 1 (1)</t>
         </is>
       </c>
       <c r="N7" s="80" t="inlineStr">
         <is>
-          <t>PASS – Business-line review/approval is supported by the BCiC manager approval fields for Claudia Romero dated 05/05/2026. Supplemental approval emails/attestations are used where available.</t>
+          <t>PASS – Business-line review/approval is supported by the BCiC manager approval fields for Claudia Romero dated 05/05/2026. Supplemental approval emails/attestations are used where available.
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 10) – Department Manager / Approval Date
+• E09 – RE: Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi</t>
         </is>
       </c>
       <c r="O7" s="80" t="inlineStr">
@@ -2751,7 +2883,7 @@
       <c r="BL7" s="61" t="n"/>
       <c r="BM7" s="61" t="n"/>
     </row>
-    <row r="8" ht="195" customFormat="1" customHeight="1" s="39">
+    <row r="8" ht="309" customFormat="1" customHeight="1" s="39">
       <c r="A8" s="45" t="n">
         <v>3299</v>
       </c>
@@ -2763,69 +2895,120 @@
 • E02 – screenshot BCiC apps in scope for DR Testing
 • E03 – All Data Integrity Validation Testing FV (row 11, 13; also 5, 51, 53, 57)
 • E05 – IT BIA Results Review and preparation for DR
-• E06 – IT BIA Results Review and preparation for DR  1 (1)
-• E14 – RE  Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) (1)
-• E16 – RE  Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 2 (1)</t>
+• E06 – IT BIA Results Review and preparation for DR 1 (1)
+• E14 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) (1)
+• E16 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 2 (1)</t>
         </is>
       </c>
       <c r="C8" s="45" t="inlineStr">
         <is>
-          <t>Imaging101</t>
+          <t>Imaging101
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 24)
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E03 – All Data Integrity Validation Testing FV (row 11, 13; also 5, 51, 53, 57)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
         </is>
       </c>
       <c r="D8" s="45" t="inlineStr">
         <is>
-          <t>Claudia Romero</t>
+          <t>Claudia Romero
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 11, 13; also 5, 51, 53, 57)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
         </is>
       </c>
       <c r="E8" s="45" t="inlineStr">
         <is>
-          <t>11/15/2025</t>
+          <t>11/15/2025
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 11, 13; also 5, 51, 53, 57)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)
+• E09 – RE: Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi</t>
         </is>
       </c>
       <c r="F8" s="45" t="inlineStr">
         <is>
-          <t>Andreina De Stefano</t>
+          <t>Andreina De Stefano
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 11, 13; also 5, 51, 53, 57)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
         </is>
       </c>
       <c r="G8" s="45" t="inlineStr">
         <is>
-          <t>Varies by record</t>
+          <t>Varies by record
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 11, 13; also 5, 51, 53, 57)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
         </is>
       </c>
       <c r="H8" s="45" t="inlineStr">
         <is>
-          <t>See source DIV procedures for Imaging101 business processes</t>
+          <t>See source DIV procedures for Imaging101 business processes
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 11, 13; also 5, 51, 53, 57) – 'Data Integrity Validation Procedures' column
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
         </is>
       </c>
       <c r="I8" s="45" t="inlineStr">
         <is>
-          <t>Yes – Client Back Office group-level approval is evidenced by Claudia Romero’s 05/05/2026 approval of the backup/restore test results. Scope mapping ties Imaging101 to Client Back Office.</t>
+          <t>Yes – Client Back Office group-level approval is evidenced by Claudia Romero’s 05/05/2026 approval of the backup/restore test results. Scope mapping ties Imaging101 to Client Back Office.
+See BSI.IT.6.C7.3 evidence folder:
+• E09 – RE: Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi
+• E14 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) (1)
+• E14a – Data Integrity Attestation Santander-BCiC (005) - BSA-AML-OFAC Compliance
+• E16 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 2 (1)
+• E16a – Data Integrity Attestation Santander-BCiC
+→ Claudia Romero – "Approved" 05/05/2026 (Client Back Office); David Marquez signed attestation 08/19/2026 (BSA/AML/OFAC Imaging101 record); M.T. Del Cerro signed attestation 08/19/2026 (Governance / MFO Imaging101 records)</t>
         </is>
       </c>
       <c r="J8" s="46" t="inlineStr">
         <is>
-          <t>VALID – BCIC evidence confirmed. The BC in the Cloud 'Data Integrity Validation Testing' screen directly displays this application and the control fields for Business Data Validation Date, Department Manager, Department Manager Approval Date, and Y/N Format, Headers, and Content. The detailed BCIC source export supports the full application record.</t>
+          <t>VALID – BCIC evidence confirmed. The BC in the Cloud 'Data Integrity Validation Testing' screen directly displays this application and the control fields for Business Data Validation Date, Department Manager, Department Manager Approval Date, and Y/N Format, Headers, and Content. The detailed BCIC source export supports the full application record.
+See BSI.IT.6.C7.3 evidence folder:
+• E04 – BCiC Screenshot for Data Integrity Validation report
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E03 – All Data Integrity Validation Testing FV
+• E01 – Applications In Scope for DR Test BSI (13)</t>
         </is>
       </c>
       <c r="K8" s="80" t="inlineStr">
         <is>
-          <t>PASS – The application is included in the annual DR/Data Integrity Validation testing population for the review period, supported by the documented 2025/2026 DR exercises and the BCiC testing records.</t>
+          <t>PASS – The application is included in the annual DR/Data Integrity Validation testing population for the review period, supported by the documented 2025/2026 DR exercises and the BCiC testing records.
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 24) – Exercise Date / 2025-2026 DR Test Scope
+• E03 – All Data Integrity Validation Testing FV (row 11, 13; also 5, 51, 53, 57) – Business Data Validation Date / Last App DR Test Date</t>
         </is>
       </c>
       <c r="L8" s="80" t="inlineStr">
         <is>
-          <t>PASS – IT DR facilitated the Data Integrity Validation process and the designated business-line tester performed the validation during the DR exercise. The application record contains the validation date/results.</t>
+          <t>PASS – IT DR facilitated the Data Integrity Validation process and the designated business-line tester performed the validation during the DR exercise. The application record contains the validation date/results.
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 11, 13; also 5, 51, 53, 57) – Y/N Format, Headers, Content = Y
+• E09 – RE: Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi</t>
         </is>
       </c>
       <c r="M8" s="80" t="inlineStr">
         <is>
-          <t>PASS – Imaging101 is supported as in scope through the BCM/BIA process led by Elizabeth Noda and corroborated by the BCiC/workpaper scope population. A separate Michael Sacilotto approval list is not required for the evidenced process. See Management_Attestation folder</t>
+          <t>PASS – Imaging101 is supported as in scope through the BCM/BIA process led by Elizabeth Noda and corroborated by the BCiC/workpaper scope population. A separate Michael Sacilotto approval list is not required for the evidenced process. See Management_Attestation folder
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 24)
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E05 – IT BIA Results Review and preparation for DR
+• E06 – IT BIA Results Review and preparation for DR 1 (1)</t>
         </is>
       </c>
       <c r="N8" s="80" t="inlineStr">
         <is>
-          <t>PASS – Business-line review/approval is supported by the BCiC manager approval fields for Andreina De Stefano dated Varies by record. Supplemental approval emails/attestations are used where available.</t>
+          <t>PASS – Business-line review/approval is supported by the BCiC manager approval fields for Andreina De Stefano dated Varies by record. Supplemental approval emails/attestations are used where available.
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 11, 13; also 5, 51, 53, 57) – Department Manager / Approval Date
+• E09 – RE: Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi
+• E14 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) (1)
+• E14a – Data Integrity Attestation Santander-BCiC (005) - BSA-AML-OFAC Compliance
+• E16 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 2 (1)
+• E16a – Data Integrity Attestation Santander-BCiC</t>
         </is>
       </c>
       <c r="O8" s="80" t="inlineStr">
@@ -2911,7 +3094,7 @@
       <c r="BL8" s="61" t="n"/>
       <c r="BM8" s="61" t="n"/>
     </row>
-    <row r="9" ht="180" customFormat="1" customHeight="1" s="39">
+    <row r="9" ht="283" customFormat="1" customHeight="1" s="39">
       <c r="A9" s="45" t="n">
         <v>4052</v>
       </c>
@@ -2923,68 +3106,111 @@
 • E02 – screenshot BCiC apps in scope for DR Testing
 • E03 – All Data Integrity Validation Testing FV (row 61)
 • E05 – IT BIA Results Review and preparation for DR
-• E06 – IT BIA Results Review and preparation for DR  1 (1)
-• E15 – RE  Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 1 (1)</t>
+• E06 – IT BIA Results Review and preparation for DR 1 (1)
+• E15 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 1 (1)</t>
         </is>
       </c>
       <c r="C9" s="45" t="inlineStr">
         <is>
-          <t>Interface Monitor</t>
+          <t>Interface Monitor
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 25)
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E03 – All Data Integrity Validation Testing FV (row 61)
+• E04 – BCiC Screenshot for Data Integrity Validation report (screen of the report; record on later page)</t>
         </is>
       </c>
       <c r="D9" s="45" t="inlineStr">
         <is>
-          <t>Michelle Oropesa</t>
+          <t>Michelle Oropesa
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 61)
+• E04 – BCiC Screenshot for Data Integrity Validation report (screen of the report; record on later page)</t>
         </is>
       </c>
       <c r="E9" s="45" t="inlineStr">
         <is>
-          <t>11/15/2025</t>
+          <t>11/15/2025
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 61)
+• E04 – BCiC Screenshot for Data Integrity Validation report (screen of the report; record on later page)</t>
         </is>
       </c>
       <c r="F9" s="45" t="inlineStr">
         <is>
-          <t>Michelle Oropesa</t>
+          <t>Michelle Oropesa
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 61)
+• E04 – BCiC Screenshot for Data Integrity Validation report (screen of the report; record on later page)</t>
         </is>
       </c>
       <c r="G9" s="45" t="inlineStr">
         <is>
-          <t>08/17/2026</t>
+          <t>08/17/2026
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 61)
+• E04 – BCiC Screenshot for Data Integrity Validation report (screen of the report; record on later page)</t>
         </is>
       </c>
       <c r="H9" s="45" t="inlineStr">
         <is>
-          <t>Treasury Hub &amp; Derivatives Operations Interface Monitor Data Integrity Validation (DIV) Procedure</t>
+          <t>Treasury Hub &amp; Derivatives Operations Interface Monitor Data Integrity Validation (DIV) Procedure
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 61) – 'Data Integrity Validation Procedures' column
+• E04 – BCiC Screenshot for Data Integrity Validation report (screen of the report; record on later page)</t>
         </is>
       </c>
       <c r="I9" s="45" t="inlineStr">
         <is>
-          <t>Yes – Michelle Oropesa returned the signed Management Attestation on 08/17/2026 (matches BCiC Department Manager Approval Date 08/17/2026). See BSI.IT.6.C7.3_E15_RE_ Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 1 (1).msg.eml</t>
+          <t>Yes – Michelle Oropesa returned the signed Management Attestation on 08/17/2026 (matches BCiC Department Manager Approval Date 08/17/2026). See BSI.IT.6.C7.3_E15_RE_ Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 1 (1).msg.eml
+See BSI.IT.6.C7.3 evidence folder:
+• E15 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 1 (1)
+• E15a – Data Integrity Attestation Santander-BCiC
+→ Michelle Oropesa – signed attestation 08/17/2026 (matches BCiC Manager Approval Date 08/17/2026)</t>
         </is>
       </c>
       <c r="J9" s="46" t="inlineStr">
         <is>
-          <t>VALID – BCIC evidence confirmed through source-report corroboration. The supplied BC in the Cloud 'Data Integrity Validation Testing' screenshot establishes the BCIC system-of-record/report used for the detailed DIV source export, and the 'Applications In Scope for DR Test BSI' screenshot corroborates the BCIC DR-scope population. The detailed export contains this application's DIV record(s), validation results, and manager approval fields.</t>
+          <t>VALID – BCIC evidence confirmed through source-report corroboration. The supplied BC in the Cloud 'Data Integrity Validation Testing' screenshot establishes the BCIC system-of-record/report used for the detailed DIV source export, and the 'Applications In Scope for DR Test BSI' screenshot corroborates the BCIC DR-scope population. The detailed export contains this application's DIV record(s), validation results, and manager approval fields.
+See BSI.IT.6.C7.3 evidence folder:
+• E04 – BCiC Screenshot for Data Integrity Validation report
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E03 – All Data Integrity Validation Testing FV
+• E01 – Applications In Scope for DR Test BSI (13)</t>
         </is>
       </c>
       <c r="K9" s="80" t="inlineStr">
         <is>
-          <t>PASS – The application is included in the annual DR/Data Integrity Validation testing population for the review period, supported by the documented 2025/2026 DR exercises and the BCiC testing records.</t>
+          <t>PASS – The application is included in the annual DR/Data Integrity Validation testing population for the review period, supported by the documented 2025/2026 DR exercises and the BCiC testing records.
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 25) – Exercise Date / 2025-2026 DR Test Scope
+• E03 – All Data Integrity Validation Testing FV (row 61) – Business Data Validation Date / Last App DR Test Date</t>
         </is>
       </c>
       <c r="L9" s="80" t="inlineStr">
         <is>
-          <t>PASS – IT DR facilitated the Data Integrity Validation process and the designated business-line tester performed the validation during the DR exercise. The application record contains the validation date/results.</t>
+          <t>PASS – IT DR facilitated the Data Integrity Validation process and the designated business-line tester performed the validation during the DR exercise. The application record contains the validation date/results.
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 61) – Y/N Format, Headers, Content = Y</t>
         </is>
       </c>
       <c r="M9" s="80" t="inlineStr">
         <is>
-          <t>PASS – Interface Monitor is supported as in scope through the BCM/BIA process led by Elizabeth Noda and corroborated by the BCiC/workpaper scope population. A separate Michael Sacilotto approval list is not required for the evidenced process. See Management_Attestation folder</t>
+          <t>PASS – Interface Monitor is supported as in scope through the BCM/BIA process led by Elizabeth Noda and corroborated by the BCiC/workpaper scope population. A separate Michael Sacilotto approval list is not required for the evidenced process. See Management_Attestation folder
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 25)
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E05 – IT BIA Results Review and preparation for DR
+• E06 – IT BIA Results Review and preparation for DR 1 (1)</t>
         </is>
       </c>
       <c r="N9" s="80" t="inlineStr">
         <is>
-          <t>PASS – Business-line review/approval is supported by the BCiC manager approval fields for Michelle Oropesa dated 08/17/2026. Supplemental approval emails/attestations are used where available.</t>
+          <t>PASS – Business-line review/approval is supported by the BCiC manager approval fields for Michelle Oropesa dated 08/17/2026. Supplemental approval emails/attestations are used where available.
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 61) – Department Manager / Approval Date
+• E15 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 1 (1)
+• E15a – Data Integrity Attestation Santander-BCiC</t>
         </is>
       </c>
       <c r="O9" s="80" t="inlineStr">
@@ -3067,7 +3293,7 @@
       <c r="BL9" s="61" t="n"/>
       <c r="BM9" s="61" t="n"/>
     </row>
-    <row r="10" ht="180" customFormat="1" customHeight="1" s="39">
+    <row r="10" ht="283" customFormat="1" customHeight="1" s="39">
       <c r="A10" s="45" t="n">
         <v>3301</v>
       </c>
@@ -3079,68 +3305,115 @@
 • E02 – screenshot BCiC apps in scope for DR Testing
 • E03 – All Data Integrity Validation Testing FV (row 25, 29)
 • E05 – IT BIA Results Review and preparation for DR
-• E06 – IT BIA Results Review and preparation for DR  1 (1)
-• E17 – RE  Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 3 (1)</t>
+• E06 – IT BIA Results Review and preparation for DR 1 (1)
+• E17 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 3 (1)</t>
         </is>
       </c>
       <c r="C10" s="45" t="inlineStr">
         <is>
-          <t>MQ Payment Monitor</t>
+          <t>MQ Payment Monitor
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 31)
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E03 – All Data Integrity Validation Testing FV (row 25, 29)
+• E04 – BCiC Screenshot for Data Integrity Validation report (screen of the report; record on later page)</t>
         </is>
       </c>
       <c r="D10" s="45" t="inlineStr">
         <is>
-          <t>Franklin Puentes</t>
+          <t>Franklin Puentes
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 25, 29)
+• E04 – BCiC Screenshot for Data Integrity Validation report (screen of the report; record on later page)</t>
         </is>
       </c>
       <c r="E10" s="45" t="inlineStr">
         <is>
-          <t>11/15/2025</t>
+          <t>11/15/2025
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 25, 29)
+• E04 – BCiC Screenshot for Data Integrity Validation report (screen of the report; record on later page)
+• E07 – DATA INTERITY FILS FROM 111425
+• E08 – FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425</t>
         </is>
       </c>
       <c r="F10" s="45" t="inlineStr">
         <is>
-          <t>Franklin Puentes</t>
+          <t>Franklin Puentes
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 25, 29)
+• E04 – BCiC Screenshot for Data Integrity Validation report (screen of the report; record on later page)</t>
         </is>
       </c>
       <c r="G10" s="45" t="inlineStr">
         <is>
-          <t>12/18/2025</t>
+          <t>12/18/2025
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 25, 29)
+• E04 – BCiC Screenshot for Data Integrity Validation report (screen of the report; record on later page)</t>
         </is>
       </c>
       <c r="H10" s="45" t="inlineStr">
         <is>
-          <t>BSI Cash Management MQ Data Integrity Validation (DIV) Procedure</t>
+          <t>BSI Cash Management MQ Data Integrity Validation (DIV) Procedure
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 25, 29) – 'Data Integrity Validation Procedures' column
+• E04 – BCiC Screenshot for Data Integrity Validation report (screen of the report; record on later page)</t>
         </is>
       </c>
       <c r="I10" s="45" t="inlineStr">
         <is>
-          <t>Yes – Frank Puentes returned the signed Management Attestation on 08/18/2026 (matches BCiC Attestation Date 08/18/2026). See BSI.IT.6.C7.3_E17_RE_ Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 3 (1).msg.eml</t>
+          <t>Yes – Frank Puentes returned the signed Management Attestation on 08/18/2026 (matches BCiC Attestation Date 08/18/2026). See BSI.IT.6.C7.3_E17_RE_ Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 3 (1).msg.eml
+See BSI.IT.6.C7.3 evidence folder:
+• E17 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 3 (1)
+• E17a – 4069 001
+→ Frank Puentes – signed attestation 08/18/2026 (matches BCiC Attestation Date 08/18/2026)</t>
         </is>
       </c>
       <c r="J10" s="46" t="inlineStr">
         <is>
-          <t>VALID – BCIC evidence confirmed through source-report corroboration. The supplied BC in the Cloud 'Data Integrity Validation Testing' screenshot establishes the BCIC system-of-record/report used for the detailed DIV source export, and the 'Applications In Scope for DR Test BSI' screenshot corroborates the BCIC DR-scope population. The detailed export contains this application's DIV record(s), validation results, and manager approval fields.</t>
+          <t>VALID – BCIC evidence confirmed through source-report corroboration. The supplied BC in the Cloud 'Data Integrity Validation Testing' screenshot establishes the BCIC system-of-record/report used for the detailed DIV source export, and the 'Applications In Scope for DR Test BSI' screenshot corroborates the BCIC DR-scope population. The detailed export contains this application's DIV record(s), validation results, and manager approval fields.
+See BSI.IT.6.C7.3 evidence folder:
+• E04 – BCiC Screenshot for Data Integrity Validation report
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E03 – All Data Integrity Validation Testing FV
+• E01 – Applications In Scope for DR Test BSI (13)</t>
         </is>
       </c>
       <c r="K10" s="80" t="inlineStr">
         <is>
-          <t>PASS – The application is included in the annual DR/Data Integrity Validation testing population for the review period, supported by the documented 2025/2026 DR exercises and the BCiC testing records.</t>
+          <t>PASS – The application is included in the annual DR/Data Integrity Validation testing population for the review period, supported by the documented 2025/2026 DR exercises and the BCiC testing records.
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 31) – Exercise Date / 2025-2026 DR Test Scope
+• E03 – All Data Integrity Validation Testing FV (row 25, 29) – Business Data Validation Date / Last App DR Test Date</t>
         </is>
       </c>
       <c r="L10" s="80" t="inlineStr">
         <is>
-          <t>PASS – IT DR facilitated the Data Integrity Validation process and the designated business-line tester performed the validation during the DR exercise. The application record contains the validation date/results.</t>
+          <t>PASS – IT DR facilitated the Data Integrity Validation process and the designated business-line tester performed the validation during the DR exercise. The application record contains the validation date/results.
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 25, 29) – Y/N Format, Headers, Content = Y
+• E07 – DATA INTERITY FILS FROM 111425
+• E08 – FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425</t>
         </is>
       </c>
       <c r="M10" s="80" t="inlineStr">
         <is>
-          <t>PASS – MQ Payment Monitor is supported as in scope through the BCM/BIA process led by Elizabeth Noda and corroborated by the BCiC/workpaper scope population. A separate Michael Sacilotto approval list is not required for the evidenced process. See Management_Attestation folder</t>
+          <t>PASS – MQ Payment Monitor is supported as in scope through the BCM/BIA process led by Elizabeth Noda and corroborated by the BCiC/workpaper scope population. A separate Michael Sacilotto approval list is not required for the evidenced process. See Management_Attestation folder
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 31)
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E05 – IT BIA Results Review and preparation for DR
+• E06 – IT BIA Results Review and preparation for DR 1 (1)</t>
         </is>
       </c>
       <c r="N10" s="80" t="inlineStr">
         <is>
-          <t>PASS – Business-line review/approval is supported by the BCiC manager approval fields for Franklin Puentes dated 12/18/2025. Supplemental approval emails/attestations are used where available.</t>
+          <t>PASS – Business-line review/approval is supported by the BCiC manager approval fields for Franklin Puentes dated 12/18/2025. Supplemental approval emails/attestations are used where available.
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 25, 29) – Department Manager / Approval Date
+• E17 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 3 (1)
+• E17a – 4069 001</t>
         </is>
       </c>
       <c r="O10" s="80" t="inlineStr">
@@ -3225,7 +3498,7 @@
       <c r="BL10" s="61" t="n"/>
       <c r="BM10" s="61" t="n"/>
     </row>
-    <row r="11" ht="195" customFormat="1" customHeight="1" s="39">
+    <row r="11" ht="309" customFormat="1" customHeight="1" s="39">
       <c r="A11" s="45" t="n">
         <v>1903</v>
       </c>
@@ -3237,69 +3510,120 @@
 • E02 – screenshot BCiC apps in scope for DR Testing
 • E03 – All Data Integrity Validation Testing FV (row 6; also 26, 30, 34, 58)
 • E05 – IT BIA Results Review and preparation for DR
-• E06 – IT BIA Results Review and preparation for DR  1 (1)
-• E14 – RE  Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) (1)
-• E17 – RE  Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 3 (1)</t>
+• E06 – IT BIA Results Review and preparation for DR 1 (1)
+• E14 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) (1)
+• E17 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 3 (1)</t>
         </is>
       </c>
       <c r="C11" s="45" t="inlineStr">
         <is>
-          <t>OFAC - BSI</t>
+          <t>OFAC - BSI
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 34)
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E03 – All Data Integrity Validation Testing FV (row 6; also 26, 30, 34, 58)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
         </is>
       </c>
       <c r="D11" s="45" t="inlineStr">
         <is>
-          <t>David Marquez</t>
+          <t>David Marquez
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 6; also 26, 30, 34, 58)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
         </is>
       </c>
       <c r="E11" s="40" t="inlineStr">
         <is>
-          <t>11/15/2025</t>
+          <t>11/15/2025
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 6; also 26, 30, 34, 58)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)
+• E07 – DATA INTERITY FILS FROM 111425
+• E08 – FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425</t>
         </is>
       </c>
       <c r="F11" s="45" t="inlineStr">
         <is>
-          <t>David Marquez</t>
-        </is>
-      </c>
-      <c r="G11" s="49" t="inlineStr">
-        <is>
-          <t>11/15/2025</t>
+          <t>David Marquez
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 6; also 26, 30, 34, 58)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
+        </is>
+      </c>
+      <c r="G11" s="82" t="inlineStr">
+        <is>
+          <t>11/15/2025
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 6; also 26, 30, 34, 58)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
         </is>
       </c>
       <c r="H11" s="40" t="inlineStr">
         <is>
-          <t>OFAC-related DIV procedures</t>
+          <t>OFAC-related DIV procedures
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 6; also 26, 30, 34, 58) – 'Data Integrity Validation Procedures' column
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
         </is>
       </c>
       <c r="I11" s="40" t="inlineStr">
         <is>
-          <t>Yes – David Marquez returned the signed Management Attestation on 08/19/2026 (BSA/AML/OFAC record); Frank Puentes signed 08/18/2026 for the Payments OFAC records. See BSI.IT.6.C7.3_E14_RE_ Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) (1).msg.eml</t>
+          <t>Yes – David Marquez returned the signed Management Attestation on 08/19/2026 (BSA/AML/OFAC record); Frank Puentes signed 08/18/2026 for the Payments OFAC records. See BSI.IT.6.C7.3_E14_RE_ Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) (1).msg.eml
+See BSI.IT.6.C7.3 evidence folder:
+• E14 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) (1)
+• E14a – Data Integrity Attestation Santander-BCiC (005) - BSA-AML-OFAC Compliance
+• E17 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 3 (1)
+• E17a – 4069 001
+→ David Marquez – signed attestation 08/19/2026 (BSA/AML/OFAC record); Frank Puentes – signed attestation 08/18/2026 (Payments OFAC records)</t>
         </is>
       </c>
       <c r="J11" s="41" t="inlineStr">
         <is>
-          <t>VALID – BCIC evidence confirmed. The BC in the Cloud 'Data Integrity Validation Testing' screen directly displays this application and the control fields for Business Data Validation Date, Department Manager, Department Manager Approval Date, and Y/N Format, Headers, and Content. The detailed BCIC source export supports the full application record.</t>
+          <t>VALID – BCIC evidence confirmed. The BC in the Cloud 'Data Integrity Validation Testing' screen directly displays this application and the control fields for Business Data Validation Date, Department Manager, Department Manager Approval Date, and Y/N Format, Headers, and Content. The detailed BCIC source export supports the full application record.
+See BSI.IT.6.C7.3 evidence folder:
+• E04 – BCiC Screenshot for Data Integrity Validation report
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E03 – All Data Integrity Validation Testing FV
+• E01 – Applications In Scope for DR Test BSI (13)</t>
         </is>
       </c>
       <c r="K11" s="80" t="inlineStr">
         <is>
-          <t>PASS – The application is included in the annual DR/Data Integrity Validation testing population for the review period, supported by the documented 2025/2026 DR exercises and the BCiC testing records.</t>
+          <t>PASS – The application is included in the annual DR/Data Integrity Validation testing population for the review period, supported by the documented 2025/2026 DR exercises and the BCiC testing records.
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 34) – Exercise Date / 2025-2026 DR Test Scope
+• E03 – All Data Integrity Validation Testing FV (row 6; also 26, 30, 34, 58) – Business Data Validation Date / Last App DR Test Date</t>
         </is>
       </c>
       <c r="L11" s="80" t="inlineStr">
         <is>
-          <t>PASS – IT DR facilitated the Data Integrity Validation process and the designated business-line tester performed the validation during the DR exercise. The application record contains the validation date/results.</t>
+          <t>PASS – IT DR facilitated the Data Integrity Validation process and the designated business-line tester performed the validation during the DR exercise. The application record contains the validation date/results.
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 6; also 26, 30, 34, 58) – Y/N Format, Headers, Content = Y
+• E07 – DATA INTERITY FILS FROM 111425
+• E08 – FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425</t>
         </is>
       </c>
       <c r="M11" s="80" t="inlineStr">
         <is>
-          <t>PASS – OFAC - BSI is supported as in scope through the BCM/BIA process led by Elizabeth Noda and corroborated by the BCiC/workpaper scope population. A separate Michael Sacilotto approval list is not required for the evidenced process. See Management_Attestation folder</t>
+          <t>PASS – OFAC - BSI is supported as in scope through the BCM/BIA process led by Elizabeth Noda and corroborated by the BCiC/workpaper scope population. A separate Michael Sacilotto approval list is not required for the evidenced process. See Management_Attestation folder
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 34)
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E05 – IT BIA Results Review and preparation for DR
+• E06 – IT BIA Results Review and preparation for DR 1 (1)</t>
         </is>
       </c>
       <c r="N11" s="80" t="inlineStr">
         <is>
-          <t>PASS – Business-line review/approval is supported by the BCiC manager approval fields for David Marquez dated 11/15/2025. Supplemental approval emails/attestations are used where available.</t>
+          <t>PASS – Business-line review/approval is supported by the BCiC manager approval fields for David Marquez dated 11/15/2025. Supplemental approval emails/attestations are used where available.
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 6; also 26, 30, 34, 58) – Department Manager / Approval Date
+• E14 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) (1)
+• E14a – Data Integrity Attestation Santander-BCiC (005) - BSA-AML-OFAC Compliance
+• E17 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 3 (1)
+• E17a – 4069 001</t>
         </is>
       </c>
       <c r="O11" s="80" t="inlineStr">
@@ -3386,7 +3710,7 @@
       <c r="BL11" s="61" t="n"/>
       <c r="BM11" s="61" t="n"/>
     </row>
-    <row r="12" ht="165" customFormat="1" customHeight="1" s="39">
+    <row r="12" ht="283" customFormat="1" customHeight="1" s="39">
       <c r="A12" s="45" t="n">
         <v>1917</v>
       </c>
@@ -3398,67 +3722,118 @@
 • E02 – screenshot BCiC apps in scope for DR Testing
 • E03 – All Data Integrity Validation Testing FV (row 17)
 • E05 – IT BIA Results Review and preparation for DR
-• E06 – IT BIA Results Review and preparation for DR  1 (1)</t>
+• E06 – IT BIA Results Review and preparation for DR 1 (1)</t>
         </is>
       </c>
       <c r="C12" s="45" t="inlineStr">
         <is>
-          <t>ReconXpert</t>
+          <t>ReconXpert
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 36)
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E03 – All Data Integrity Validation Testing FV (row 17)
+• E04 – BCiC Screenshot for Data Integrity Validation report (screen of the report; record on later page)</t>
         </is>
       </c>
       <c r="D12" s="45" t="inlineStr">
         <is>
-          <t>Sadis Alvarenga Hernandez|Dunia Gonzalez Collado</t>
+          <t>Sadis Alvarenga Hernandez|Dunia Gonzalez Collado
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 17)
+• E04 – BCiC Screenshot for Data Integrity Validation report (screen of the report; record on later page)</t>
         </is>
       </c>
       <c r="E12" s="45" t="inlineStr">
         <is>
-          <t>11/15/2025</t>
+          <t>11/15/2025
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 17)
+• E04 – BCiC Screenshot for Data Integrity Validation report (screen of the report; record on later page)
+• E10 – RE: Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert
+• E11 – BSI.IT.6.C7.3 Manager Approval
+• E12 – RE: Testing enviroment Financial Analysis manager approval</t>
         </is>
       </c>
       <c r="F12" s="45" t="inlineStr">
         <is>
-          <t>Sadis Alvarenga Hernandez</t>
+          <t>Sadis Alvarenga Hernandez
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 17)
+• E04 – BCiC Screenshot for Data Integrity Validation report (screen of the report; record on later page)</t>
         </is>
       </c>
       <c r="G12" s="45" t="inlineStr">
         <is>
-          <t>01/26/2026</t>
+          <t>01/26/2026
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 17)
+• E04 – BCiC Screenshot for Data Integrity Validation report (screen of the report; record on later page)</t>
         </is>
       </c>
       <c r="H12" s="45" t="inlineStr">
         <is>
-          <t>General ledger review ReconXpert Data Integrity Validation (DIV) Procedure</t>
+          <t>General ledger review ReconXpert Data Integrity Validation (DIV) Procedure
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 17) – 'Data Integrity Validation Procedures' column
+• E04 – BCiC Screenshot for Data Integrity Validation report (screen of the report; record on later page)</t>
         </is>
       </c>
       <c r="I12" s="45" t="inlineStr">
         <is>
-          <t>Yes – Finance group-level approval is evidenced by Lina Acuna’s 03/09/2026 approval. The scope email maps ReconXpert to Financial Analysis and Control.</t>
+          <t>Yes – Finance group-level approval is evidenced by Lina Acuna’s 03/09/2026 approval. The scope email maps ReconXpert to Financial Analysis and Control.
+See BSI.IT.6.C7.3 evidence folder:
+• E12 – RE: Testing enviroment Financial Analysis manager approval
+• E10 – RE: Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert
+• E11 – BSI.IT.6.C7.3 Manager Approval
+→ Sadis Alvarenga – "Approved" 01/26/2026 (matches BCiC Manager Approval Date 01/26/2026); Lina Acuna – Finance "Approved" 03/09/2026 with DIV chart</t>
         </is>
       </c>
       <c r="J12" s="44" t="inlineStr">
         <is>
-          <t>VALID – BCIC evidence confirmed through source-report corroboration. The supplied BC in the Cloud 'Data Integrity Validation Testing' screenshot establishes the BCIC system-of-record/report used for the detailed DIV source export, and the 'Applications In Scope for DR Test BSI' screenshot corroborates the BCIC DR-scope population. The detailed export contains this application's DIV record(s), validation results, and manager approval fields.</t>
+          <t>VALID – BCIC evidence confirmed through source-report corroboration. The supplied BC in the Cloud 'Data Integrity Validation Testing' screenshot establishes the BCIC system-of-record/report used for the detailed DIV source export, and the 'Applications In Scope for DR Test BSI' screenshot corroborates the BCIC DR-scope population. The detailed export contains this application's DIV record(s), validation results, and manager approval fields.
+See BSI.IT.6.C7.3 evidence folder:
+• E04 – BCiC Screenshot for Data Integrity Validation report
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E03 – All Data Integrity Validation Testing FV
+• E01 – Applications In Scope for DR Test BSI (13)</t>
         </is>
       </c>
       <c r="K12" s="80" t="inlineStr">
         <is>
-          <t>PASS – The application is included in the annual DR/Data Integrity Validation testing population for the review period, supported by the documented 2025/2026 DR exercises and the BCiC testing records.</t>
+          <t>PASS – The application is included in the annual DR/Data Integrity Validation testing population for the review period, supported by the documented 2025/2026 DR exercises and the BCiC testing records.
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 36) – Exercise Date / 2025-2026 DR Test Scope
+• E03 – All Data Integrity Validation Testing FV (row 17) – Business Data Validation Date / Last App DR Test Date</t>
         </is>
       </c>
       <c r="L12" s="80" t="inlineStr">
         <is>
-          <t>PASS – IT DR facilitated the Data Integrity Validation process and the designated business-line tester performed the validation during the DR exercise. The application record contains the validation date/results.</t>
+          <t>PASS – IT DR facilitated the Data Integrity Validation process and the designated business-line tester performed the validation during the DR exercise. The application record contains the validation date/results.
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 17) – Y/N Format, Headers, Content = Y
+• E10 – RE: Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert
+• E11 – BSI.IT.6.C7.3 Manager Approval
+• E12 – RE: Testing enviroment Financial Analysis manager approval</t>
         </is>
       </c>
       <c r="M12" s="80" t="inlineStr">
         <is>
-          <t>PASS – ReconXpert is supported as in scope through the BCM/BIA process led by Elizabeth Noda and corroborated by the BCiC/workpaper scope population. A separate Michael Sacilotto approval list is not required for the evidenced process. See Management_Attestation folder</t>
+          <t>PASS – ReconXpert is supported as in scope through the BCM/BIA process led by Elizabeth Noda and corroborated by the BCiC/workpaper scope population. A separate Michael Sacilotto approval list is not required for the evidenced process. See Management_Attestation folder
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 36)
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E05 – IT BIA Results Review and preparation for DR
+• E06 – IT BIA Results Review and preparation for DR 1 (1)</t>
         </is>
       </c>
       <c r="N12" s="80" t="inlineStr">
         <is>
-          <t>PASS – Business-line review/approval is supported by the BCiC manager approval fields for Sadis Alvarenga Hernandez dated 01/26/2026. Supplemental approval emails/attestations are used where available.</t>
+          <t>PASS – Business-line review/approval is supported by the BCiC manager approval fields for Sadis Alvarenga Hernandez dated 01/26/2026. Supplemental approval emails/attestations are used where available.
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 17) – Department Manager / Approval Date
+• E12 – RE: Testing enviroment Financial Analysis manager approval
+• E10 – RE: Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert
+• E11 – BSI.IT.6.C7.3 Manager Approval</t>
         </is>
       </c>
       <c r="O12" s="80" t="inlineStr">
@@ -3542,7 +3917,7 @@
       <c r="BL12" s="61" t="n"/>
       <c r="BM12" s="61" t="n"/>
     </row>
-    <row r="13" ht="195" customFormat="1" customHeight="1" s="39">
+    <row r="13" ht="309" customFormat="1" customHeight="1" s="39">
       <c r="A13" s="45" t="n">
         <v>1936</v>
       </c>
@@ -3554,69 +3929,120 @@
 • E02 – screenshot BCiC apps in scope for DR Testing
 • E03 – All Data Integrity Validation Testing FV (row 7; also 60)
 • E05 – IT BIA Results Review and preparation for DR
-• E06 – IT BIA Results Review and preparation for DR  1 (1)
-• E14 – RE  Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) (1)
-• E15 – RE  Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 1 (1)</t>
+• E06 – IT BIA Results Review and preparation for DR 1 (1)
+• E14 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) (1)
+• E15 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 1 (1)</t>
         </is>
       </c>
       <c r="C13" s="45" t="inlineStr">
         <is>
-          <t>Swift Interface - BSI</t>
-        </is>
-      </c>
-      <c r="D13" s="49" t="inlineStr">
-        <is>
-          <t>David Marquez</t>
+          <t>Swift Interface - BSI
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 42)
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E03 – All Data Integrity Validation Testing FV (row 7; also 60)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
+        </is>
+      </c>
+      <c r="D13" s="82" t="inlineStr">
+        <is>
+          <t>David Marquez
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 7; also 60)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
         </is>
       </c>
       <c r="E13" s="45" t="inlineStr">
         <is>
-          <t>11/15/2025</t>
-        </is>
-      </c>
-      <c r="F13" s="49" t="inlineStr">
-        <is>
-          <t>David Marquez</t>
+          <t>11/15/2025
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 7; also 60)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)
+• E07 – DATA INTERITY FILS FROM 111425
+• E08 – FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425</t>
+        </is>
+      </c>
+      <c r="F13" s="82" t="inlineStr">
+        <is>
+          <t>David Marquez
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 7; also 60)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
         </is>
       </c>
       <c r="G13" s="45" t="inlineStr">
         <is>
-          <t>11/15/2025</t>
+          <t>11/15/2025
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 7; also 60)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
         </is>
       </c>
       <c r="H13" s="40" t="inlineStr">
         <is>
-          <t>Swift Interface - BSI Data Integrity Validation (DIV) Procedure</t>
+          <t>Swift Interface - BSI Data Integrity Validation (DIV) Procedure
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 7; also 60) – 'Data Integrity Validation Procedures' column
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
         </is>
       </c>
       <c r="I13" s="40" t="inlineStr">
         <is>
-          <t>Yes – David Marquez signed attestation 08/19/2026 (BSA/AML/OFAC record) and Michelle Oropesa signed attestation 08/17/2026 (Investment Ops record). See BSI.IT.6.C7.3_E14_RE_ Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) (1).msg.eml</t>
+          <t>Yes – David Marquez signed attestation 08/19/2026 (BSA/AML/OFAC record) and Michelle Oropesa signed attestation 08/17/2026 (Investment Ops record). See BSI.IT.6.C7.3_E14_RE_ Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) (1).msg.eml
+See BSI.IT.6.C7.3 evidence folder:
+• E14 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) (1)
+• E14a – Data Integrity Attestation Santander-BCiC (005) - BSA-AML-OFAC Compliance
+• E15 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 1 (1)
+• E15a – Data Integrity Attestation Santander-BCiC
+→ David Marquez – signed attestation 08/19/2026 (BSA/AML/OFAC record); Michelle Oropesa – signed attestation 08/17/2026 (Investment Ops record)</t>
         </is>
       </c>
       <c r="J13" s="41" t="inlineStr">
         <is>
-          <t>VALID – BCIC evidence confirmed. The BC in the Cloud 'Data Integrity Validation Testing' screen directly displays this application and the control fields for Business Data Validation Date, Department Manager, Department Manager Approval Date, and Y/N Format, Headers, and Content. The detailed BCIC source export supports the full application record.</t>
+          <t>VALID – BCIC evidence confirmed. The BC in the Cloud 'Data Integrity Validation Testing' screen directly displays this application and the control fields for Business Data Validation Date, Department Manager, Department Manager Approval Date, and Y/N Format, Headers, and Content. The detailed BCIC source export supports the full application record.
+See BSI.IT.6.C7.3 evidence folder:
+• E04 – BCiC Screenshot for Data Integrity Validation report
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E03 – All Data Integrity Validation Testing FV
+• E01 – Applications In Scope for DR Test BSI (13)</t>
         </is>
       </c>
       <c r="K13" s="80" t="inlineStr">
         <is>
-          <t>PASS – The application is included in the annual DR/Data Integrity Validation testing population for the review period, supported by the documented 2025/2026 DR exercises and the BCiC testing records.</t>
+          <t>PASS – The application is included in the annual DR/Data Integrity Validation testing population for the review period, supported by the documented 2025/2026 DR exercises and the BCiC testing records.
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 42) – Exercise Date / 2025-2026 DR Test Scope
+• E03 – All Data Integrity Validation Testing FV (row 7; also 60) – Business Data Validation Date / Last App DR Test Date</t>
         </is>
       </c>
       <c r="L13" s="80" t="inlineStr">
         <is>
-          <t>PASS – IT DR facilitated the Data Integrity Validation process and the designated business-line tester performed the validation during the DR exercise. The application record contains the validation date/results.</t>
+          <t>PASS – IT DR facilitated the Data Integrity Validation process and the designated business-line tester performed the validation during the DR exercise. The application record contains the validation date/results.
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 7; also 60) – Y/N Format, Headers, Content = Y
+• E07 – DATA INTERITY FILS FROM 111425
+• E08 – FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425</t>
         </is>
       </c>
       <c r="M13" s="80" t="inlineStr">
         <is>
-          <t>PASS – Swift Interface - BSI is supported as in scope through the BCM/BIA process led by Elizabeth Noda and corroborated by the BCiC/workpaper scope population. A separate Michael Sacilotto approval list is not required for the evidenced process. See Management_Attestation folder</t>
+          <t>PASS – Swift Interface - BSI is supported as in scope through the BCM/BIA process led by Elizabeth Noda and corroborated by the BCiC/workpaper scope population. A separate Michael Sacilotto approval list is not required for the evidenced process. See Management_Attestation folder
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 42)
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E05 – IT BIA Results Review and preparation for DR
+• E06 – IT BIA Results Review and preparation for DR 1 (1)</t>
         </is>
       </c>
       <c r="N13" s="80" t="inlineStr">
         <is>
-          <t>PASS – Business-line review/approval is supported by the BCiC manager approval fields for David Marquez dated 11/15/2025. Supplemental approval emails/attestations are used where available.</t>
+          <t>PASS – Business-line review/approval is supported by the BCiC manager approval fields for David Marquez dated 11/15/2025. Supplemental approval emails/attestations are used where available.
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 7; also 60) – Department Manager / Approval Date
+• E14 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) (1)
+• E14a – Data Integrity Attestation Santander-BCiC (005) - BSA-AML-OFAC Compliance
+• E15 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 1 (1)
+• E15a – Data Integrity Attestation Santander-BCiC</t>
         </is>
       </c>
       <c r="O13" s="80" t="inlineStr">
@@ -3703,7 +4129,7 @@
       <c r="BL13" s="61" t="n"/>
       <c r="BM13" s="61" t="n"/>
     </row>
-    <row r="14" ht="225" customFormat="1" customHeight="1" s="39">
+    <row r="14" ht="409" customFormat="1" customHeight="1" s="39">
       <c r="A14" s="43" t="n">
         <v>1937</v>
       </c>
@@ -3715,71 +4141,136 @@
 • E02 – screenshot BCiC apps in scope for DR Testing
 • E03 – All Data Integrity Validation Testing FV (row 2 (AIS – sampled record); T24 appears on 30 records)
 • E05 – IT BIA Results Review and preparation for DR
-• E06 – IT BIA Results Review and preparation for DR  1 (1)
-• E14 – RE  Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) (1)
-• E15 – RE  Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 1 (1)
-• E16 – RE  Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 2 (1)
-• E17 – RE  Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 3 (1)</t>
+• E06 – IT BIA Results Review and preparation for DR 1 (1)
+• E14 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) (1)
+• E15 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 1 (1)
+• E16 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 2 (1)
+• E17 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 3 (1)</t>
         </is>
       </c>
       <c r="C14" s="43" t="inlineStr">
         <is>
-          <t>T24</t>
-        </is>
-      </c>
-      <c r="D14" s="50" t="inlineStr">
-        <is>
-          <t>Alfonso Camano</t>
+          <t>T24
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 43)
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E03 – All Data Integrity Validation Testing FV (row 2 (AIS – sampled record); T24 appears on 30 records)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
+        </is>
+      </c>
+      <c r="D14" s="83" t="inlineStr">
+        <is>
+          <t>Alfonso Camano
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 2 (AIS – sampled record); T24 appears on 30 records)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
         </is>
       </c>
       <c r="E14" s="43" t="inlineStr">
         <is>
-          <t>11/15/2025</t>
+          <t>11/15/2025
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 2 (AIS – sampled record); T24 appears on 30 records)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)
+• E10 – RE: Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert
+• E11 – BSI.IT.6.C7.3 Manager Approval
+• E13 – miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly</t>
         </is>
       </c>
       <c r="F14" s="43" t="inlineStr">
         <is>
-          <t>Ricardo Garcia</t>
-        </is>
-      </c>
-      <c r="G14" s="63" t="inlineStr">
-        <is>
-          <t>08/18/2026</t>
+          <t>Ricardo Garcia
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 2 (AIS – sampled record); T24 appears on 30 records)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
+        </is>
+      </c>
+      <c r="G14" s="83" t="inlineStr">
+        <is>
+          <t>08/18/2026
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 2 (AIS – sampled record); T24 appears on 30 records)
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
         </is>
       </c>
       <c r="H14" s="43" t="inlineStr">
         <is>
-          <t>Corresponding T24 DIV procedures by business process</t>
+          <t>Corresponding T24 DIV procedures by business process
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 2 (AIS – sampled record); T24 appears on 30 records) – 'Data Integrity Validation Procedures' column
+• E04 – BCiC Screenshot for Data Integrity Validation report (record visible)</t>
         </is>
       </c>
       <c r="I14" s="43" t="inlineStr">
         <is>
-          <t>Yes – Finance group-level approval is evidenced by Lina Acuna’s 03/09/2026 approval. The scope email maps T24 to Financial Analysis and Control.</t>
+          <t>Yes – Finance group-level approval is evidenced by Lina Acuna’s 03/09/2026 approval. The scope email maps T24 to Financial Analysis and Control.
+See BSI.IT.6.C7.3 evidence folder:
+• E10 – RE: Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert
+• E11 – BSI.IT.6.C7.3 Manager Approval
+• E14 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) (1)
+• E14a – Data Integrity Attestation Santander-BCiC (005) - BSA-AML-OFAC Compliance
+• E15 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 1 (1)
+• E15a – Data Integrity Attestation Santander-BCiC
+• E16 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 2 (1)
+• E16a – Data Integrity Attestation Santander-BCiC
+• E17 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 3 (1)
+• E17a – 4069 001
+→ Sampled manager Ricardo Garcia: approval 08/18/2026 evidenced in BCiC (E03/E04) – no standalone email from R. Garcia in package. Other T24 business lines: Lina Acuna 03/09/2026, D. Marquez 08/19/2026, M. Oropesa 08/17/2026, M.T. Del Cerro 08/19/2026, F. Puentes 08/18/2026</t>
         </is>
       </c>
       <c r="J14" s="44" t="inlineStr">
         <is>
-          <t>VALID – BCIC evidence confirmed. The BC in the Cloud 'Data Integrity Validation Testing' screen directly displays this application and the control fields for Business Data Validation Date, Department Manager, Department Manager Approval Date, and Y/N Format, Headers, and Content. The detailed BCIC source export supports the full application record.</t>
+          <t>VALID – BCIC evidence confirmed. The BC in the Cloud 'Data Integrity Validation Testing' screen directly displays this application and the control fields for Business Data Validation Date, Department Manager, Department Manager Approval Date, and Y/N Format, Headers, and Content. The detailed BCIC source export supports the full application record.
+See BSI.IT.6.C7.3 evidence folder:
+• E04 – BCiC Screenshot for Data Integrity Validation report
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E03 – All Data Integrity Validation Testing FV
+• E01 – Applications In Scope for DR Test BSI (13)</t>
         </is>
       </c>
       <c r="K14" s="80" t="inlineStr">
         <is>
-          <t>PASS – The application is included in the annual DR/Data Integrity Validation testing population for the review period, supported by the documented 2025/2026 DR exercises and the BCiC testing records.</t>
+          <t>PASS – The application is included in the annual DR/Data Integrity Validation testing population for the review period, supported by the documented 2025/2026 DR exercises and the BCiC testing records.
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 43) – Exercise Date / 2025-2026 DR Test Scope
+• E03 – All Data Integrity Validation Testing FV (row 2 (AIS – sampled record); T24 appears on 30 records) – Business Data Validation Date / Last App DR Test Date</t>
         </is>
       </c>
       <c r="L14" s="80" t="inlineStr">
         <is>
-          <t>PASS – IT DR facilitated the Data Integrity Validation process and the designated business-line tester performed the validation during the DR exercise. The application record contains the validation date/results.</t>
+          <t>PASS – IT DR facilitated the Data Integrity Validation process and the designated business-line tester performed the validation during the DR exercise. The application record contains the validation date/results.
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 2 (AIS – sampled record); T24 appears on 30 records) – Y/N Format, Headers, Content = Y
+• E10 – RE: Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert
+• E11 – BSI.IT.6.C7.3 Manager Approval
+• E13 – miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly</t>
         </is>
       </c>
       <c r="M14" s="80" t="inlineStr">
         <is>
-          <t>PASS – T24 is supported as in scope through the BCM/BIA process led by Elizabeth Noda and corroborated by the BCiC/workpaper scope population. A separate Michael Sacilotto approval list is not required for the evidenced process. See Management_Attestation folder</t>
+          <t>PASS – T24 is supported as in scope through the BCM/BIA process led by Elizabeth Noda and corroborated by the BCiC/workpaper scope population. A separate Michael Sacilotto approval list is not required for the evidenced process. See Management_Attestation folder
+See BSI.IT.6.C7.3 evidence folder:
+• E01 – Applications In Scope for DR Test BSI (13) (row 43)
+• E02 – screenshot BCiC apps in scope for DR Testing
+• E05 – IT BIA Results Review and preparation for DR
+• E06 – IT BIA Results Review and preparation for DR 1 (1)</t>
         </is>
       </c>
       <c r="N14" s="80" t="inlineStr">
         <is>
-          <t>PASS – Business-line review/approval is supported by the BCiC manager approval fields for Ricardo Garcia dated 08/18/2026. Supplemental approval emails/attestations are used where available.</t>
+          <t>PASS – Business-line review/approval is supported by the BCiC manager approval fields for Ricardo Garcia dated 08/18/2026. Supplemental approval emails/attestations are used where available.
+See BSI.IT.6.C7.3 evidence folder:
+• E03 – All Data Integrity Validation Testing FV (row 2 (AIS – sampled record); T24 appears on 30 records) – Department Manager / Approval Date
+• E10 – RE: Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert
+• E11 – BSI.IT.6.C7.3 Manager Approval
+• E14 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) (1)
+• E14a – Data Integrity Attestation Santander-BCiC (005) - BSA-AML-OFAC Compliance
+• E15 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 1 (1)
+• E15a – Data Integrity Attestation Santander-BCiC
+• E16 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 2 (1)
+• E16a – Data Integrity Attestation Santander-BCiC
+• E17 – RE: Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 3 (1)
+• E17a – 4069 001</t>
         </is>
       </c>
       <c r="O14" s="80" t="inlineStr">
@@ -6565,7 +7056,7 @@
       <c r="A17" t="n">
         <v>1</v>
       </c>
-      <c r="B17" s="82" t="inlineStr">
+      <c r="B17" s="83" t="inlineStr">
         <is>
           <t>Imaging101 (Sample 3299): the workpaper shows Business Tester = Claudia Romero and Manager = Andreina De Stefano. BCiC (E03 rows 11/13) shows Tester = Andreina De Stefano / Rolando Bonilla and Department Manager = Claudia Romero (approval 05/05/2026). Names appear swapped – please confirm.</t>
         </is>
@@ -6575,7 +7066,7 @@
       <c r="A18" t="n">
         <v>2</v>
       </c>
-      <c r="B18" s="82" t="inlineStr">
+      <c r="B18" s="83" t="inlineStr">
         <is>
           <t>FedExport - BSI (Sample 1867): BCiC Manager Approval Date is 06/05/2026 (E03 row 9, E04) while Claudia Romero's approval email is dated 05/05/2026 (E09) and FedImport/ACH Express show 05/05/2026 – likely a BCiC data-entry date; approval still after the 11/15/2025 validation.</t>
         </is>
@@ -6585,7 +7076,7 @@
       <c r="A19" t="n">
         <v>3</v>
       </c>
-      <c r="B19" s="82" t="inlineStr">
+      <c r="B19" s="83" t="inlineStr">
         <is>
           <t>Interface Monitor, MQ Payment Monitor, OFAC - BSI and Swift Interface - BSI were previously marked 'No' for approval emails. The Management Attestation emails (E14/E15/E17 with signed PDFs E14a/E15a/E17a) evidence the business-line manager approval – column I updated accordingly.</t>
         </is>
@@ -6595,7 +7086,7 @@
       <c r="A20" t="n">
         <v>4</v>
       </c>
-      <c r="B20" s="82" t="inlineStr">
+      <c r="B20" s="83" t="inlineStr">
         <is>
           <t>T24 (Sample 1937): the sampled BCiC record (AIS) is approved by Ricardo Garcia 08/18/2026 in BCiC (E03 row 2 / E04). No standalone email from Ricardo Garcia is in the evidence package; other T24 business lines are covered by E10/E11, E14–E17.</t>
         </is>
@@ -6605,7 +7096,7 @@
       <c r="A21" t="n">
         <v>5</v>
       </c>
-      <c r="B21" s="82" t="inlineStr">
+      <c r="B21" s="83" t="inlineStr">
         <is>
           <t>Duplicates not retained in the evidence folder (identical files): 'RE_ Yearly Backup and restore exercise- client back office sign off.msg' (= E09) and 'RE_ Yearly Backup and restore exercise-- re-run- Finance approval.msg' (= E10).</t>
         </is>
@@ -6615,7 +7106,7 @@
       <c r="A22" t="n">
         <v>6</v>
       </c>
-      <c r="B22" s="82" t="inlineStr">
+      <c r="B22" s="83" t="inlineStr">
         <is>
           <t>E13 (T24 environment refresh, 11/13/2024) is outside the 08/01/2025–06/01/2026 review period – supplemental only.</t>
         </is>

</xml_diff>